<commit_message>
formats + sheet fidelity: csv and image extractors, workbook styling, cell selection
- xlsx v2 captures styling meta (bold/fills/colors, number formats, column
  widths, merges, frozen panes) via a size-capped second parse; page_meta
  registry table; styling is display context, never citation identity
- evidence carries sheet meta and per-window styles; spec + legend updated
- artifact renders workbook styling in cell windows and the full-sheet view,
  with Excel number formats, real column widths, and click-to-select cells
  with a name box
- csv/tsv extractor: one-sheet workbook, A1 refs, dialect sniffing
- image extractor (png/jpeg/tiff) through the vision model; the file is its
  own stored snapshot; auto selection degrades with a specific nudge
- demo workbook styled and artifact regenerated (identical tokens); roadmap
  graduates built items; 0.3.0

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo/sources/underwriting-model.xlsx
+++ b/demo/sources/underwriting-model.xlsx
@@ -17,8 +17,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+  </numFmts>
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,14 +31,26 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <color rgb="FF0000CC"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E79"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -50,11 +65,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -472,16 +495,16 @@
       <c r="B2" t="n">
         <v>44</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="2" t="n">
         <v>712</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="3" t="n">
         <v>1395</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="3" t="n">
         <v>1465</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="4" t="n">
         <v>0.955</v>
       </c>
     </row>
@@ -494,16 +517,16 @@
       <c r="B3" t="n">
         <v>38</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="2" t="n">
         <v>918</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="3" t="n">
         <v>1640</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="3" t="n">
         <v>1725</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="4" t="n">
         <v>0.947</v>
       </c>
     </row>
@@ -516,16 +539,16 @@
       <c r="B4" t="n">
         <v>32</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="2" t="n">
         <v>1042</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="3" t="n">
         <v>1835</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="3" t="n">
         <v>1930</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="4" t="n">
         <v>0.9379999999999999</v>
       </c>
     </row>
@@ -538,38 +561,38 @@
       <c r="B5" t="n">
         <v>14</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="2" t="n">
         <v>1268</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="3" t="n">
         <v>2140</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="3" t="n">
         <v>2245</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="4" t="n">
         <v>0.929</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Total / Weighted Avg</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="5" t="n">
         <v>128</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7" s="5" t="n">
         <v>916</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="5" t="n">
         <v>1659</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="5" t="n">
         <v>1744</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="6" t="n">
         <v>0.946</v>
       </c>
     </row>
@@ -579,7 +602,7 @@
           <t>Gross potential rent (annual)</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" s="3" t="n">
         <v>2972160</v>
       </c>
     </row>
@@ -589,7 +612,7 @@
           <t>Economic occupancy (T12)</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B10" s="4" t="n">
         <v>0.903</v>
       </c>
     </row>
@@ -599,7 +622,7 @@
           <t>Effective gross income</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B11" s="3" t="n">
         <v>2684400</v>
       </c>
     </row>
@@ -653,7 +676,7 @@
           <t>Going-in cap rate</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="7" t="n">
         <v>0.0575</v>
       </c>
       <c r="C2" t="inlineStr">
@@ -673,7 +696,7 @@
           <t>Exit cap rate</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="7" t="n">
         <v>0.0625</v>
       </c>
       <c r="C3" t="inlineStr">
@@ -693,7 +716,7 @@
           <t>Hold period</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="8" t="n">
         <v>5</v>
       </c>
       <c r="C4" t="inlineStr">
@@ -713,7 +736,7 @@
           <t>Rent growth, year 1</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="7" t="n">
         <v>0.032</v>
       </c>
       <c r="C5" t="inlineStr">
@@ -733,7 +756,7 @@
           <t>Rent growth, years 2-5</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="7" t="n">
         <v>0.028</v>
       </c>
       <c r="C6" t="inlineStr">
@@ -753,7 +776,7 @@
           <t>Expense growth</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="7" t="n">
         <v>0.03</v>
       </c>
       <c r="C7" t="inlineStr">
@@ -773,7 +796,7 @@
           <t>Vacancy and credit loss</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" s="7" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="C8" t="inlineStr">
@@ -793,7 +816,7 @@
           <t>Replacement reserve</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" s="9" t="n">
         <v>250</v>
       </c>
       <c r="C9" t="inlineStr">
@@ -813,7 +836,7 @@
           <t>Purchase price</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B10" s="9" t="n">
         <v>24850000</v>
       </c>
       <c r="C10" t="inlineStr">
@@ -833,7 +856,7 @@
           <t>Loan amount</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B11" s="9" t="n">
         <v>16152500</v>
       </c>
       <c r="C11" t="inlineStr">
@@ -853,7 +876,7 @@
           <t>Interest rate</t>
         </is>
       </c>
-      <c r="B12" t="n">
+      <c r="B12" s="7" t="n">
         <v>0.0615</v>
       </c>
       <c r="C12" t="inlineStr">
@@ -873,7 +896,7 @@
           <t>Amortization</t>
         </is>
       </c>
-      <c r="B13" t="n">
+      <c r="B13" s="8" t="n">
         <v>30</v>
       </c>
       <c r="C13" t="inlineStr">
@@ -893,7 +916,7 @@
           <t>Year 1 NOI (underwritten)</t>
         </is>
       </c>
-      <c r="B14" t="n">
+      <c r="B14" s="9" t="n">
         <v>1487400</v>
       </c>
       <c r="C14" t="inlineStr">
@@ -913,7 +936,7 @@
           <t>Year 1 DSCR</t>
         </is>
       </c>
-      <c r="B15" t="n">
+      <c r="B15" s="8" t="n">
         <v>1.34</v>
       </c>
       <c r="C15" t="inlineStr">
@@ -933,7 +956,7 @@
           <t>Going-in yield on cost</t>
         </is>
       </c>
-      <c r="B16" t="n">
+      <c r="B16" s="7" t="n">
         <v>0.0599</v>
       </c>
       <c r="C16" t="inlineStr">

</xml_diff>